<commit_message>
add Longest consecutive problem
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780EBEDD-6AC9-4C5A-B47F-AFBB8E3B7D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC3BE49-4286-4E04-A32E-039B9AB6662F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -4365,9 +4365,11 @@
         <v>76</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G12" s="2">
+        <v>40</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>77</v>
       </c>
@@ -9586,7 +9588,7 @@
       </c>
       <c r="D12" s="2" t="str">
         <f>'DSA Problems'!F12</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>

</xml_diff>

<commit_message>
added MaximumsumSubarray and MaximumAverageSubarray
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F46F43F-AFAD-4017-8772-62300F7B79E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{486F7E66-F734-4146-8B64-987D2B381DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -4867,9 +4867,11 @@
         <v>76</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G29" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G29" s="2">
+        <v>30</v>
+      </c>
       <c r="H29" s="2" t="s">
         <v>77</v>
       </c>
@@ -4895,9 +4897,11 @@
         <v>76</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G30" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G30" s="2">
+        <v>30</v>
+      </c>
       <c r="H30" s="2" t="s">
         <v>77</v>
       </c>
@@ -10017,7 +10021,7 @@
       </c>
       <c r="D29" s="2" t="str">
         <f>'DSA Problems'!F29</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -10042,7 +10046,7 @@
       </c>
       <c r="D30" s="2" t="str">
         <f>'DSA Problems'!F30</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>

</xml_diff>

<commit_message>
added Longest Substring without repeatingChar
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{486F7E66-F734-4146-8B64-987D2B381DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{535BAFBF-784A-43A0-977A-9B899E56499A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -4927,9 +4927,11 @@
         <v>76</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G31" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G31" s="2">
+        <v>40</v>
+      </c>
       <c r="H31" s="2" t="s">
         <v>77</v>
       </c>
@@ -10071,7 +10073,7 @@
       </c>
       <c r="D31" s="2" t="str">
         <f>'DSA Problems'!F31</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>

</xml_diff>

<commit_message>
Added Find All Anagrams in string
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FDA038-68A8-43FE-866E-6BE04D32275C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350E8E1C-918D-4577-AC8E-7378D5371051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -4987,9 +4987,11 @@
         <v>76</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G33" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G33" s="2">
+        <v>40</v>
+      </c>
       <c r="H33" s="2" t="s">
         <v>77</v>
       </c>
@@ -5015,9 +5017,11 @@
         <v>76</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G34" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G34" s="2">
+        <v>40</v>
+      </c>
       <c r="H34" s="2" t="s">
         <v>77</v>
       </c>
@@ -5043,7 +5047,7 @@
         <v>76</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2" t="s">
@@ -10125,7 +10129,7 @@
       </c>
       <c r="D33" s="2" t="str">
         <f>'DSA Problems'!F33</f>
-        <v>In Progress</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -10150,7 +10154,7 @@
       </c>
       <c r="D34" s="2" t="str">
         <f>'DSA Problems'!F34</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -10175,7 +10179,7 @@
       </c>
       <c r="D35" s="2" t="str">
         <f>'DSA Problems'!F35</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>

</xml_diff>

<commit_message>
added Minimum Window SubString
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209BE3FA-7978-4802-9796-D024DE127AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E95F12C-E015-40B7-98C2-05ED20D1944F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -5077,9 +5077,11 @@
         <v>76</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G36" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G36" s="2">
+        <v>45</v>
+      </c>
       <c r="H36" s="2" t="s">
         <v>77</v>
       </c>
@@ -10206,7 +10208,7 @@
       </c>
       <c r="D36" s="2" t="str">
         <f>'DSA Problems'!F36</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>

</xml_diff>

<commit_message>
added prefix suffix sum problems
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{691AA9C9-7C66-4B5A-86C2-B25DEB5D8791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EB1B43-E643-46E7-9A31-E0807B2B8FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1830" uniqueCount="253">
   <si>
     <t>DSA 90-Day Interview Preparation Dashboard</t>
   </si>
@@ -795,6 +795,9 @@
   </si>
   <si>
     <t>it cannot be executed local</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I have to relearn it</t>
   </si>
 </sst>
 </file>
@@ -1220,7 +1223,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -5167,9 +5170,11 @@
         <v>76</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G39" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G39" s="2">
+        <v>25</v>
+      </c>
       <c r="H39" s="2" t="s">
         <v>77</v>
       </c>
@@ -5264,7 +5269,9 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
+      <c r="L42" s="2" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
@@ -5283,9 +5290,11 @@
         <v>118</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G43" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G43" s="2">
+        <v>25</v>
+      </c>
       <c r="H43" s="2" t="s">
         <v>77</v>
       </c>
@@ -5311,9 +5320,11 @@
         <v>118</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G44" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G44" s="2">
+        <v>25</v>
+      </c>
       <c r="H44" s="2" t="s">
         <v>77</v>
       </c>
@@ -5339,9 +5350,11 @@
         <v>118</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G45" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G45" s="2">
+        <v>25</v>
+      </c>
       <c r="H45" s="2" t="s">
         <v>77</v>
       </c>
@@ -5367,9 +5380,11 @@
         <v>118</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G46" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G46" s="2">
+        <v>25</v>
+      </c>
       <c r="H46" s="2" t="s">
         <v>77</v>
       </c>
@@ -10291,7 +10306,7 @@
       </c>
       <c r="D39" s="2" t="str">
         <f>'DSA Problems'!F39</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
@@ -10391,7 +10406,7 @@
       </c>
       <c r="D43" s="2" t="str">
         <f>'DSA Problems'!F43</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
@@ -10416,7 +10431,7 @@
       </c>
       <c r="D44" s="2" t="str">
         <f>'DSA Problems'!F44</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
@@ -10441,7 +10456,7 @@
       </c>
       <c r="D45" s="2" t="str">
         <f>'DSA Problems'!F45</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
@@ -10466,7 +10481,7 @@
       </c>
       <c r="D46" s="2" t="str">
         <f>'DSA Problems'!F46</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>

</xml_diff>

<commit_message>
added fast api basics
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EB1B43-E643-46E7-9A31-E0807B2B8FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B865D4-0A08-497B-BBE1-6751FB20B068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added binary search problesms
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B865D4-0A08-497B-BBE1-6751FB20B068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBA2AE1-9003-4D48-9447-CD962ED2EB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -5556,9 +5556,11 @@
         <v>76</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G52" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G52" s="2">
+        <v>20</v>
+      </c>
       <c r="H52" s="2" t="s">
         <v>77</v>
       </c>
@@ -5584,9 +5586,11 @@
         <v>76</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G53" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G53" s="2">
+        <v>20</v>
+      </c>
       <c r="H53" s="2" t="s">
         <v>77</v>
       </c>
@@ -5612,9 +5616,11 @@
         <v>76</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G54" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G54" s="2">
+        <v>20</v>
+      </c>
       <c r="H54" s="2" t="s">
         <v>77</v>
       </c>
@@ -10631,7 +10637,7 @@
       </c>
       <c r="D52" s="2" t="str">
         <f>'DSA Problems'!F52</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
@@ -10656,7 +10662,7 @@
       </c>
       <c r="D53" s="2" t="str">
         <f>'DSA Problems'!F53</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
@@ -10681,7 +10687,7 @@
       </c>
       <c r="D54" s="2" t="str">
         <f>'DSA Problems'!F54</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>

</xml_diff>

<commit_message>
added binary search problems
</commit_message>
<xml_diff>
--- a/documents/plan/DSA_90_Day_Roadmap.xlsx
+++ b/documents/plan/DSA_90_Day_Roadmap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SreenivasReddyDaram\Target-learn\documents\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBA2AE1-9003-4D48-9447-CD962ED2EB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9076C9D-C0D1-4E1C-8F3B-579A55A77725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('DSA Problems'!F:F,"Needs Revision")</f>
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -5646,9 +5646,11 @@
         <v>76</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G55" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G55" s="2">
+        <v>20</v>
+      </c>
       <c r="H55" s="2" t="s">
         <v>77</v>
       </c>
@@ -5674,9 +5676,11 @@
         <v>76</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G56" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="G56" s="2">
+        <v>20</v>
+      </c>
       <c r="H56" s="2" t="s">
         <v>77</v>
       </c>
@@ -10712,7 +10716,7 @@
       </c>
       <c r="D55" s="2" t="str">
         <f>'DSA Problems'!F55</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
@@ -10737,7 +10741,7 @@
       </c>
       <c r="D56" s="2" t="str">
         <f>'DSA Problems'!F56</f>
-        <v>Not Started</v>
+        <v>Needs Revision</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>

</xml_diff>